<commit_message>
update data, improve some code
</commit_message>
<xml_diff>
--- a/Data/Data-sheet.xlsx
+++ b/Data/Data-sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tristancools/Documents/Arduino/Project-experimenteren2/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{574319FD-C77A-C747-B259-37068857164B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8D504D27-61F0-5A4F-A6EB-ABD0E63ADA92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="21000" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kalibratie" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="55">
   <si>
     <t>d(cm)</t>
   </si>
@@ -265,6 +265,9 @@
   </si>
   <si>
     <t>Foutpercentage</t>
+  </si>
+  <si>
+    <t>AF (dtheta)</t>
   </si>
 </sst>
 </file>
@@ -4145,13 +4148,14 @@
     <col min="9" max="9" width="8.33203125" customWidth="1"/>
     <col min="10" max="10" width="8" customWidth="1"/>
     <col min="11" max="11" width="7.83203125" customWidth="1"/>
-    <col min="12" max="13" width="8.33203125" customWidth="1"/>
+    <col min="12" max="12" width="8.33203125" customWidth="1"/>
+    <col min="13" max="13" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="19.5" customWidth="1"/>
-    <col min="15" max="16" width="16.6640625" customWidth="1"/>
-    <col min="17" max="17" width="19" customWidth="1"/>
-    <col min="18" max="18" width="18" customWidth="1"/>
-    <col min="19" max="19" width="17.6640625" customWidth="1"/>
-    <col min="20" max="20" width="20.1640625" customWidth="1"/>
+    <col min="15" max="15" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="13" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="18" customWidth="1"/>
     <col min="22" max="22" width="17.6640625" customWidth="1"/>
   </cols>
@@ -4192,7 +4196,7 @@
         <v>45</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="N1" s="3" t="s">
         <v>22</v>

</xml_diff>